<commit_message>
Turn most of the listing template into dropdowns
Free typing produced Faraya three different ways in the last import. The town list is the 60 already in the directory.
</commit_message>
<xml_diff>
--- a/vardenia-listing-template.xlsx
+++ b/vardenia-listing-template.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me first" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +34,9 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -88,23 +92,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -470,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -523,83 +528,79 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Category and District are dropdowns. Use them. A category typed by hand that is not</t>
+          <t>Most columns are dropdowns - click the cell and a little arrow appears. Use them.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>on the list means the row is rejected, and the list is short because it matches the</t>
+          <t>Only the business name, the activity and the description have to be typed.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>sections that exist on the site.</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Category, District, Hotel Stars and Usually When will refuse anything not on the list,</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Only Mount Lebanon for now</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>because a value off the list cannot be imported at all.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>The importer currently covers Keserwan and Byblos / Jbeil only. A business anywhere</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>else needs a change to the site first - send it separately rather than inventing a district.</t>
+          <t>Location and Price Range only warn. If a village is genuinely not on the list, type it</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>and carry on. Otherwise pick the one that is there - Faraya typed three different ways</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Photos</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>becomes three different places on the site.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Do not put photos in this file. Photos go in folders, one folder per business.</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>After this sheet is filled in, run scripts/make-photo-folders.mjs and it creates the</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Only Mount Lebanon for now</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>empty folders for you, named correctly, with a note in each saying what goes inside.</t>
+          <t>The importer currently covers Keserwan and Byblos / Jbeil only. A business anywhere</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>You then drop the photos in and send the whole folder back.</t>
+          <t>else needs a change to the site first - send it separately rather than inventing a district.</t>
         </is>
       </c>
     </row>
@@ -607,47 +608,47 @@
       <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Inside each folder:</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Photos</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cover.jpg    the main photo, the one that appears at the top of the listing</t>
+          <t>Do not put photos in this file. Photos go in folders, one folder per business.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    01.jpg       gallery photos, in the order you want them shown</t>
+          <t>Send this sheet back first. We then send you a folder tree - one empty folder per</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    02.jpg</t>
+          <t>business, already named, with a note inside saying what goes in it. Drop the photos</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>into the folders and send the whole thing back.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Send cover plus one gallery photo unless you have been told otherwise. Listings on the</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>free tier display one gallery image, so anything beyond that is stored and never seen.</t>
+          <t>Do not rename the folders. The name is how each photo finds its listing.</t>
         </is>
       </c>
     </row>
@@ -657,36 +658,84 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Photographs must be ones we are allowed to publish. Send the credit and where each</t>
+          <t>Inside each folder:</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>came from with the folder - a photo we cannot show is worse than no photo.</t>
+          <t xml:space="preserve">    cover.jpg    the main photo, the one that appears at the top of the listing</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    01.jpg       gallery photos, in the order you want them shown</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>What happens to what you write</t>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    02.jpg</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Nothing appears on the site automatically. Every listing arrives as a draft and somebody</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
+        <is>
+          <t>Send cover plus one gallery photo unless you have been told otherwise. Listings on the</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>free tier display one gallery image, so anything beyond that is stored and never seen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Photographs must be ones we are allowed to publish. Send the credit and where each</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>came from with the folder - a photo we cannot show is worse than no photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>What happens to what you write</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Nothing appears on the site automatically. Every listing arrives as a draft and somebody</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>on the team reads it before it is published.</t>
         </is>
@@ -788,7 +837,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Town or village. Goes on the listing as its address.</t>
+          <t>Town or village. Pick from the list; type a new one only if it is genuinely not there.</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -798,17 +847,17 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Hotels only. 1 to 5. Under 4 files the hotel as boutique rather than luxury.</t>
+          <t>Hotels only. Pick 1 to 5. Under 4 files the hotel as boutique rather than luxury.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Write it with a dollar sign, for example $80 or $80-120. Banded automatically.</t>
+          <t>Pick the band a typical visit or night costs.</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>The Google rating, 0 to 5, one decimal. Leave empty if you have not checked.</t>
+          <t>The Google rating, 0 to 5. Leave empty if you have not checked it.</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -851,7 +900,7 @@
       <c r="F3" s="6" t="inlineStr"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>$90-140</t>
+          <t>$50-149</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -878,17 +927,474 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Not an accepted value" error="Pick one of the listed options. Anything else is rejected by the importer." prompt="Choose from the list" type="list">
+  <dataValidations count="7">
+    <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not an accepted value" error="Pick one of the listed options - anything else is rejected by the importer." type="list" errorStyle="stop">
       <formula1>"Hotels,Guest Houses,Restaurants,Activities,Tour Guides,Festivals"</formula1>
     </dataValidation>
-    <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Not an accepted value" error="Pick one of the listed options. Anything else is rejected by the importer." prompt="Choose from the list" type="list">
+    <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not an accepted value" error="Pick one of the listed options - anything else is rejected by the importer." type="list" errorStyle="stop">
       <formula1>"Keserwan District,Byblos / Jbeil District,Keserwan + Byblos / Jbeil Districts"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Not an accepted value" error="Pick one of the listed options. Anything else is rejected by the importer." prompt="Choose from the list" type="list">
+    <dataValidation sqref="D3:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="That is not on the list. Continue only if it is genuinely a new one." type="list" errorStyle="warning">
+      <formula1>Lists!$A$2:$A$61</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an accepted value" error="Pick one of the listed options - anything else is rejected by the importer." type="list" errorStyle="stop">
+      <formula1>"1,2,3,4,5"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="That is not on the list. Continue only if it is genuinely a new one." type="list" errorStyle="warning">
+      <formula1>"$0-49,$50-149,$150-299,$300+"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a rating" error="A Google rating is a number between 0 and 5, for example 4.6." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an accepted value" error="Pick one of the listed options - anything else is rejected by the importer." type="list" errorStyle="stop">
       <formula1>"Year-round,Summer,Winter,Summer and Winter"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Towns already in the directory</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aaqoura</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Adonis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ajaltoun</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Blat</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Byblos</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bzoummar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chabrouh</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Chouwen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Daraaoun</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ehmej</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Faitroun</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Faqra</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Faraya</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fatqa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Fatre</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ghalboun</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ghazir</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ghbaleh</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ghedress</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ghineh</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Halat</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Harissa</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Heart of Byblos</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hjoula</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jbeil</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Jeita</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Jounieh</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jounieh area</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Jounieh ↔️ Harissa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Kaslik</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Keserwen</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Keserwen + Jbeil Private Tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Keserwen – additional</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Kfar Yassine</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kfardebian</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Kfarehbab</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kfarhbab</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Kfaryassine</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Kfour</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Laqlouq</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mastita</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mayrouba</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Mechmech</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Nabaa Saouma</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nahr El Dahab</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Nahr Ibrahim</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Nahr Ibrahim area</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Okaibeh</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Old City</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Qahmez</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Qartaboun</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Safra</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Sahel Alma</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Saint Challita Street</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Sarba</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tabarja</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Yahchouch</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Zouk</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Zouk Mikael</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Zouk Mosbeh</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>